<commit_message>
Etiopia: zawodnicy z Kuwejtu (Transfermarkt nie ma lig kuwejckich - brak linku do ligi nie oznacza tam amatorow; NACJE[..]["kraje_bez_lig"], tylko dla Etiopii) - Kenean Markneh (Al-Arabi), Gathouch Panom (Al Fahaheel); kod kraju Kuwejtu, zeby katarskie Al-Arabi sie nie dopasowywalo
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/zawodnicy_et.xlsx
+++ b/zawodnicy_et.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -447,6 +447,40 @@
       <c r="C2" t="inlineStr">
         <is>
           <t>[Andora] Club Esportiu Carroi</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Kenean</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Markneh</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>[Kuwejt] Al-Arabi</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Gathouch</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Panom</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>[Kuwejt] Al Fahaheel</t>
         </is>
       </c>
     </row>

</xml_diff>